<commit_message>
Update app, scraper, and data files
</commit_message>
<xml_diff>
--- a/shopify_partners.xlsx
+++ b/shopify_partners.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -512,6 +512,326 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>JD1 Studio</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.jd1.co/</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>hola@jd1.co</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>57 310 501 3818</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Bogota,Colombia</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/josedan1el</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>btodigital</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://btodigital.com/</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>cbetancur@btodigital.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>+573014915522</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Medellín,Colombia</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/btodigital</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Novacode Webgency | Colombia | Miami | Panamá</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://beacons.ai/novacode</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>novacode.colombia@gmail.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>3204663232</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Medellín,Colombia</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/pablo-uzuriaga</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Jump Digital Commerce - Colombia, US, Ecuador, Chile, B2B, International</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://jumpdigital.co/</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>contact@jumpdigital.co</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>+573005587333 - +13127525924</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Bogota,Colombia</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/jump-digital2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BOTEROMEDIA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.boteromedia.com/</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>carlosandres@botero.net.co</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>+15557309292</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BOGOTÁ,Colombia</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/botero-media1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DODO Solutions</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://dodosolutions.com/</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>hello@dodosolutions.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>3006184994</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Medellín,Colombia</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/dodo-solutions</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Moxie Digital</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://moxiedigital.co/</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>info@moxiedigital.co</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>+573136491785</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Medellin,Colombia</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/moxiedigital</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Growtide</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://growtide.co/</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>carlos@growtide.co</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>+573103731555</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Medellín,Colombia</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/growtide</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ED Enlaces Digitales</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://enlacesdigitales.co/</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>gerencia@enlacesdigitales.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>+573156877912</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Bogota,Colombia</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/enlaces-digitales</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Jhon Studio</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://jhonstudio.com/</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>info@jhonstudio.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>3180363003</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Medellin,Colombia</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>https://www.shopify.com/partners/directory/partner/jhon-studio</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>